<commit_message>
feat: sync revised Excel Perubahan 2 - update HPP Rp 691.250, selling price Rp 1.000.000, PGN gas Rp 173.880, and rotary drum 4-9 RPM
</commit_message>
<xml_diff>
--- a/Database_Simulasi_SCADA_dan_Operasional.xlsx
+++ b/Database_Simulasi_SCADA_dan_Operasional.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\am878\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project Pak Heru\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ADEC9BA-12B7-4EDE-AF3E-74178AF4F8AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C208982-A3D3-4923-9CE6-29BCCC80F98E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daftar &amp; Kamus Data" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="biaya_siklus_hpp" sheetId="7" r:id="rId7"/>
     <sheet name="insiden_downtime_bottleneck" sheetId="8" r:id="rId8"/>
     <sheet name="rekap_kinerja_eksekutif" sheetId="9" r:id="rId9"/>
+    <sheet name="simulasi_skenario_demand_range" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="648">
   <si>
     <t>DATABASE OPERASIONAL &amp; TELEMETRI SCADA</t>
   </si>
@@ -1392,20 +1393,613 @@
   </si>
   <si>
     <t>biaya_maintenance_per_ton_rp</t>
+  </si>
+  <si>
+    <t>SIMULASI RENTANG DEMAND, KAPASITAS LOGISTIK TRUK, FINANSIAL, &amp; DINAMIKA INDUSTRI LOKAL</t>
+  </si>
+  <si>
+    <t>PT. MINERAL ADITIF NUSANTARA — Model Simulasi Dinamis Rentang Output (80T - 420T/Hari), 6 Skenario Lonjakan Permintaan Swasta &amp; Megaproyek Pemerintah</t>
+  </si>
+  <si>
+    <t>BAGIAN 1: MATRIKS 6 SKENARIO RENTANG DEMAND &amp; KEBUTUHAN LOGISTIK TRUK (@ 30 TON)</t>
+  </si>
+  <si>
+    <t>Kode Skenario</t>
+  </si>
+  <si>
+    <t>Nama Skenario Permintaan</t>
+  </si>
+  <si>
+    <t>Tipe Operasional / Shift</t>
+  </si>
+  <si>
+    <t>Jam Kerja Efektif</t>
+  </si>
+  <si>
+    <t>Output Harian (Ton)</t>
+  </si>
+  <si>
+    <t>Output Bulanan (25 Hari)</t>
+  </si>
+  <si>
+    <t>Rit Truk Outbound (@30T)</t>
+  </si>
+  <si>
+    <t>Rit Dibulatkan Outbound</t>
+  </si>
+  <si>
+    <t>Bentonite 80% (Ton)</t>
+  </si>
+  <si>
+    <t>Rit Truk Inbound Bentonite</t>
+  </si>
+  <si>
+    <t>Calsium 15% (Ton)</t>
+  </si>
+  <si>
+    <t>Soda Ash 5% (Ton)</t>
+  </si>
+  <si>
+    <t>Total Rit Inbound/Hari</t>
+  </si>
+  <si>
+    <t>Total Lalu Lintas Truk/Hari</t>
+  </si>
+  <si>
+    <t>Ketahanan Stockpile Bentonite (Jam)</t>
+  </si>
+  <si>
+    <t>Buffer Holding Time Silo (Jam)</t>
+  </si>
+  <si>
+    <t>Status Risiko Logistik &amp; Buffer</t>
+  </si>
+  <si>
+    <t>SCN-01</t>
+  </si>
+  <si>
+    <t>Low Demand (Pasar Kontraksi / Retail Turun)</t>
+  </si>
+  <si>
+    <t>0.5 Shift (Setengah Hari)</t>
+  </si>
+  <si>
+    <t>Sangat Aman (Turnover Lambat)</t>
+  </si>
+  <si>
+    <t>SCN-02</t>
+  </si>
+  <si>
+    <t>Normal Baseline (Standar 1 Shift Eksisting)</t>
+  </si>
+  <si>
+    <t>1 Shift Reguler (08:30-16:30)</t>
+  </si>
+  <si>
+    <t>Ideal &amp; Stabil (Ekuilibrium Pabrik)</t>
+  </si>
+  <si>
+    <t>SCN-03</t>
+  </si>
+  <si>
+    <t>High Commercial Surge (Lonjakan Swasta / Q2-Q3)</t>
+  </si>
+  <si>
+    <t>1 Shift + Lembur Maksimal 3 Jam</t>
+  </si>
+  <si>
+    <t>Moderat (Wajib Jadwal Ketat Truk)</t>
+  </si>
+  <si>
+    <t>SCN-04</t>
+  </si>
+  <si>
+    <t>Corporate Multiplier (Tender Swasta Besar / 2x)</t>
+  </si>
+  <si>
+    <t>2 Shift Penuh (07:00-23:00)</t>
+  </si>
+  <si>
+    <t>Ketat (Stockpile Habis dlm 4,2 Jam)</t>
+  </si>
+  <si>
+    <t>SCN-05</t>
+  </si>
+  <si>
+    <t>Massive Peak Tender (Proyek BUMN Karya / 2.5x)</t>
+  </si>
+  <si>
+    <t>2 Shift Panjang + 4 Jam Lembur</t>
+  </si>
+  <si>
+    <t>Tinggi (Jembatan Timbang Non-Stop)</t>
+  </si>
+  <si>
+    <t>SCN-06</t>
+  </si>
+  <si>
+    <t>Government Megaproject Surge (PSN / IKN 24 Jam)</t>
+  </si>
+  <si>
+    <t>3 Shift Kontinu (24 Jam Non-Stop)</t>
+  </si>
+  <si>
+    <t>Kritis &amp; Ekstrem (Wajib Jumbo Bag Buffer)</t>
+  </si>
+  <si>
+    <t>BAGIAN 2: STRUKTUR HPP, OMZET, LABA KOTOR, DAN KEBUTUHAN MODAL KERJA CASH FLOW (TOP 30, 60, 90 HARI)</t>
+  </si>
+  <si>
+    <t>Output Harian</t>
+  </si>
+  <si>
+    <t>Biaya Raw Material</t>
+  </si>
+  <si>
+    <t>Biaya Gas PGN</t>
+  </si>
+  <si>
+    <t>Biaya Listrik PLN</t>
+  </si>
+  <si>
+    <t>Biaya Solar Forklift</t>
+  </si>
+  <si>
+    <t>Alokasi SDM / Hari</t>
+  </si>
+  <si>
+    <t>Biaya Maintenance</t>
+  </si>
+  <si>
+    <t>Total Biaya Harian (HPP)</t>
+  </si>
+  <si>
+    <t>HPP per Ton</t>
+  </si>
+  <si>
+    <t>Harga Jual per Ton</t>
+  </si>
+  <si>
+    <t>Omzet Penjualan Harian</t>
+  </si>
+  <si>
+    <t>Laba Kotor Harian</t>
+  </si>
+  <si>
+    <t>Gross Margin Pct</t>
+  </si>
+  <si>
+    <t>Laba Kotor Bulanan (25H)</t>
+  </si>
+  <si>
+    <t>Kebutuhan Modal Kerja (TOP 30H - Swasta)</t>
+  </si>
+  <si>
+    <t>Kebutuhan Modal Kerja (TOP 60H - BUMN Menengah)</t>
+  </si>
+  <si>
+    <t>Kebutuhan Modal Kerja (TOP 90H - Tender Pemerintah)</t>
+  </si>
+  <si>
+    <t>BAGIAN 3: ANALISIS DINAMIKA INDUSTRI LOKAL INDONESIA &amp; STRATEGI MITIGASI RISIKO OPERASIONAL</t>
+  </si>
+  <si>
+    <t>Faktor Dinamika Lokal</t>
+  </si>
+  <si>
+    <t>Deskripsi Kejadian Riil di Lapangan</t>
+  </si>
+  <si>
+    <t>Dampak Langsung ke SCADA / Plant</t>
+  </si>
+  <si>
+    <t>Sensitivitas Angka / Batasan</t>
+  </si>
+  <si>
+    <t>Skenario Terdampak</t>
+  </si>
+  <si>
+    <t>SOP &amp; Strategi Mitigasi Teruji</t>
+  </si>
+  <si>
+    <t>Regulasi Jam Masuk Truk &amp; Jalur Tol Arteri</t>
+  </si>
+  <si>
+    <t>Pembatasan truk sumbu 3 / tronton di jalan tol &amp; arteri pada jam sibuk (06:00-09:00 &amp; 16:00-19:00 WIB) serta larangan angkutan barang saat libur Nataru dan Lebaran oleh Kemenhub.</t>
+  </si>
+  <si>
+    <t>Truk bahan mentah tertahan di luar area industri, menyebabkan stockpile bentonite menipis mendadak di tengah produksi.</t>
+  </si>
+  <si>
+    <t>Buffer stockpile bentonite (134,4 T) hanya bertahan 4,0 s.d. 8,4 jam operasional saat pabrik digeber penuh.</t>
+  </si>
+  <si>
+    <t>SCN-03 s.d. SCN-06</t>
+  </si>
+  <si>
+    <t>Jadwal penerimaan inbound digeser ke malam hari (22:00 - 05:00 WIB) menggunakan sistem reservasi barcode logistik terpadu.</t>
+  </si>
+  <si>
+    <t>Penegakan Kebijakan Zero ODOL (Over Dimension Over Load)</t>
+  </si>
+  <si>
+    <t>Penertiban jembatan timbang Kemenhub secara ketat membatasi muatan bersih truk tronton maksimal 30 Ton netto per ritase.</t>
+  </si>
+  <si>
+    <t>Pabrik tidak dapat memadatkan muatan menjadi 40-45 Ton/truk. Frekuensi armada truk di jalan raya wajib meningkat drastis.</t>
+  </si>
+  <si>
+    <t>Butuh 14 rit truk outbound + 15 rit inbound per hari pada Skenario 6 (Total 29 rit truk melintas di jembatan timbang internal).</t>
+  </si>
+  <si>
+    <t>SCN-04, SCN-05, SCN-06</t>
+  </si>
+  <si>
+    <t>Kemitraan multi-transporter (minimal 3 konsorsium ekspedisi terverifikasi) dan standardisasi jembatan timbang internal EQ-WB-01.</t>
+  </si>
+  <si>
+    <t>Fluktuasi Cuaca Musim Hujan (Wet Season Tambang Open Pit)</t>
+  </si>
+  <si>
+    <t>Tambang bentonite di Pulau Jawa merupakan tambang terbuka (open-pit). Saat musim hujan (Okt-Mar), kadar air (moisture) bahan mentah melonjak dari 18% ke 32-35%.</t>
+  </si>
+  <si>
+    <t>Beban termal rotary dryer naik signifikan, konsumsi gas PGN naik 15-20%, serta risiko penyumbatan (choked) pada vibrating screen &amp; conveyor.</t>
+  </si>
+  <si>
+    <t>Konsumsi PGN naik dari 6,8 MMBTU/jam ke 8,2 MMBTU/jam (Tambahan beban gas ~Rp 1,5 Juta - Rp 2,2 Juta/hari).</t>
+  </si>
+  <si>
+    <t>Semua Skenario (SCN-01 s.d. SCN-06)</t>
+  </si>
+  <si>
+    <t>Pemasangan atap terpal kanopi ganda di Stockpile Yard 1 &amp; 2 serta kontrol suhu burner otomatis modulasi SCADA.</t>
+  </si>
+  <si>
+    <t>Keterbatasan Buffer Bin Silo (72 m³ / 86,4 T) &amp; Bottleneck Bay</t>
+  </si>
+  <si>
+    <t>Bin Silo produk akhir hanya memiliki volume 72 m³. Pada kapasitas puncak 420 Ton/hari, silo penuh hanya dalam waktu 4,1 jam jika truk tangki terlambat merapat.</t>
+  </si>
+  <si>
+    <t>Silo blockage high-level alarm menyala, memaksa rotary dryer dimatikan darurat (risiko bahan bakar terbuang &amp; reheat burner Rp 17,2 - 20,5 Juta).</t>
+  </si>
+  <si>
+    <t>Loading bay harus melayani 1 rit truk tangki curah (30 Ton) setiap 85 s.d. 90 menit tanpa jeda sedikit pun.</t>
+  </si>
+  <si>
+    <t>Penerapan sistem Staging Buffer Jumbo Bag 1 Ton (PK-JMB-07) di gudang samping dengan kapasitas buffer darurat 200 Ton.</t>
+  </si>
+  <si>
+    <t>Term of Payment (TOP) Pengadaan Pemerintah &amp; BUMN Karya (60-90 Hari)</t>
+  </si>
+  <si>
+    <t>Proyek infrastruktur pemerintah (KemenPUPR, IKN, BUMN Karya) memiliki siklus pencairan 60 s.d. 90 hari setelah BAST dan verifikasi laboratorium terbit.</t>
+  </si>
+  <si>
+    <t>Cash flow gap: Pembelian bahan baku tunai/tempo 14 hari dan tagihan gas PGN jatuh tempo tgl 20, sedangkan piutang tertahan puluhan miliar rupiah.</t>
+  </si>
+  <si>
+    <t>Kebutuhan modal kerja mencapai Rp 61 Miliar (SCN-04) hingga Rp 144,1 Miliar (SCN-06) per siklus 90 hari pemesanan masif.</t>
+  </si>
+  <si>
+    <t>Mewajibkan Down Payment (DP) tender 20-30%, memanfaatkan fasilitas perbankan Supply Chain Financing (SCF) / SKBDN, dan negosiasi tempo tambang.</t>
+  </si>
+  <si>
+    <t>Regulasi Ketenagakerjaan (Batas Lembur &amp; Skema Multi-Shift)</t>
+  </si>
+  <si>
+    <t>UU Cipta Kerja No. 11/2020 &amp; PP 35/2021 membatasi kerja lembur maksimal 4 jam/hari dan 18 jam/minggu untuk melindungi K3 operator.</t>
+  </si>
+  <si>
+    <t>Operasional di atas 10 jam kerja per hari TIDAK BOLEH hanya mengandalkan lembur 1 shift, melainkan WAJIB membuka Shift 2 atau Shift 3.</t>
+  </si>
+  <si>
+    <t>Biaya SDM naik dari Rp 2,67 Juta/hari (1 Shift) menjadi Rp 5,61 Juta (2 Shift) dan Rp 9,84 Juta (3 Shift 4 regu rotasi).</t>
+  </si>
+  <si>
+    <t>Rekrutmen tenaga kerja musiman bersertifikasi K3 dan penerapan skema roster kerja 3 shift 4 regu rotasi (siklus 6 hari kerja 2 hari off).</t>
+  </si>
+  <si>
+    <t>Stres Termal &amp; Keausan Mekis Mesin Rotary Drum Dryer Kontinu</t>
+  </si>
+  <si>
+    <t>Rotary Dryer berputar pada suhu 220°C. Operasional terus menerus 21 jam/hari menyebabkan keausan bearing roll dan pemuaian refractory brick furnace.</t>
+  </si>
+  <si>
+    <t>Risiko breakdown fatal akibat bearing overheat jika tidak ada jeda pendinginan dan pelumasan teratur.</t>
+  </si>
+  <si>
+    <t>Kehilangan output 20 Ton/jam dan biaya downtime mekanis hingga puluhan juta rupiah.</t>
+  </si>
+  <si>
+    <t>SCN-05, SCN-06</t>
+  </si>
+  <si>
+    <t>Menyisakan jeda 3 jam per hari (1 jam per pergantian shift) untuk inspeksi thermal gun, re-greasing suhu tinggi, dan pembersihan filter baghouse.</t>
+  </si>
+  <si>
+    <t>Keterbatasan Ketersediaan Truk Ekspedisi Pihak Ketiga (3PL Deficit)</t>
+  </si>
+  <si>
+    <t>Pada bulan-bulan puncak proyek konstruksi nasional, permintaan truk tronton tangki dan bak curah di pasar logistik lokal melonjak drastis.</t>
+  </si>
+  <si>
+    <t>Kelangkaan armada truk sewa yang siap melayani ritase harian tepat waktu.</t>
+  </si>
+  <si>
+    <t>Terjadi penumpukan produk jadi di silo pabrik dan denda penalti keterlambatan pengiriman ke lokasi proyek pemerintah.</t>
+  </si>
+  <si>
+    <t>Menjalin kontrak eksklusif jangka panjang (Dedicated Fleet SLA) dengan 3 perusahaan logistik berbeda dengan jaminan denda penggantian armada.</t>
+  </si>
+  <si>
+    <t>BAGIAN 4: SIMULASI JADWAL DISPATCH LOGISTIK PEAK DAY (TIMELINE PER JAM: 07:00 - 23:00 WIB)</t>
+  </si>
+  <si>
+    <t>Jam (WIB)</t>
+  </si>
+  <si>
+    <t>Status Operasional SCADA</t>
+  </si>
+  <si>
+    <t>Inbound Truk Masuk (Bahan)</t>
+  </si>
+  <si>
+    <t>Outbound Truk Keluar (Produk)</t>
+  </si>
+  <si>
+    <t>Tonase Masuk (T)</t>
+  </si>
+  <si>
+    <t>Tonase Keluar (T)</t>
+  </si>
+  <si>
+    <t>Level Stockpile Bentonite (T)</t>
+  </si>
+  <si>
+    <t>Level Bin Silo (T)</t>
+  </si>
+  <si>
+    <t>Aktivitas Jembatan Timbang EQ-WB-01</t>
+  </si>
+  <si>
+    <t>Catatan Kontrol Logistik</t>
+  </si>
+  <si>
+    <t>07:00 - 08:00</t>
+  </si>
+  <si>
+    <t>Shift 1 Start / Preheating Burner</t>
+  </si>
+  <si>
+    <t>Truk Inbound 1 (Bentonite)</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Timbang Masuk Inbound 1</t>
+  </si>
+  <si>
+    <t>Stok awal bentonite 100T terisi truk malam</t>
+  </si>
+  <si>
+    <t>08:00 - 09:00</t>
+  </si>
+  <si>
+    <t>Produksi Aktif (20 Ton/Jam)</t>
+  </si>
+  <si>
+    <t>Truk Inbound 2 (Bentonite)</t>
+  </si>
+  <si>
+    <t>Truk Outbound 1 (30 Ton)</t>
+  </si>
+  <si>
+    <t>Timbang Inbound 2 &amp; Outbound 1</t>
+  </si>
+  <si>
+    <t>Ritme loading tangki produk pertama lancar</t>
+  </si>
+  <si>
+    <t>09:00 - 10:00</t>
+  </si>
+  <si>
+    <t>Truk Inbound 3 (Calsium)</t>
+  </si>
+  <si>
+    <t>Timbang Inbound 3 (Calsium)</t>
+  </si>
+  <si>
+    <t>Calsium dibongkar di Stockpile Bay 2</t>
+  </si>
+  <si>
+    <t>10:00 - 11:00</t>
+  </si>
+  <si>
+    <t>Truk Inbound 4 (Bentonite)</t>
+  </si>
+  <si>
+    <t>Truk Outbound 2 (30 Ton)</t>
+  </si>
+  <si>
+    <t>Timbang Inbound 4 &amp; Outbound 2</t>
+  </si>
+  <si>
+    <t>Stockpile bentonite terjaga di atas 120 Ton</t>
+  </si>
+  <si>
+    <t>11:00 - 12:00</t>
+  </si>
+  <si>
+    <t>Truk Inbound 5 (Soda Ash)</t>
+  </si>
+  <si>
+    <t>Timbang Inbound 5 (Soda Ash)</t>
+  </si>
+  <si>
+    <t>Dosing tank soda ash terisi penuh</t>
+  </si>
+  <si>
+    <t>12:00 - 13:00</t>
+  </si>
+  <si>
+    <t>Rotasi Shift / Istirahat Parsial</t>
+  </si>
+  <si>
+    <t>Truk Outbound 3 (30 Ton)</t>
+  </si>
+  <si>
+    <t>Timbang Outbound 3</t>
+  </si>
+  <si>
+    <t>Burner low fire standby, loading bay tetap jalan</t>
+  </si>
+  <si>
+    <t>13:00 - 14:00</t>
+  </si>
+  <si>
+    <t>Truk Inbound 6 (Bentonite)</t>
+  </si>
+  <si>
+    <t>Timbang Inbound 6 (Bentonite)</t>
+  </si>
+  <si>
+    <t>Pasokan siang masuk tepat waktu</t>
+  </si>
+  <si>
+    <t>14:00 - 15:00</t>
+  </si>
+  <si>
+    <t>Truk Outbound 4 (30 Ton)</t>
+  </si>
+  <si>
+    <t>Timbang Outbound 4</t>
+  </si>
+  <si>
+    <t>Pengiriman 120 Ton pertama tercapai</t>
+  </si>
+  <si>
+    <t>15:00 - 16:00</t>
+  </si>
+  <si>
+    <t>Shift 2 Handover / Inspeksi Mesin</t>
+  </si>
+  <si>
+    <t>Truk Inbound 7 (Bentonite)</t>
+  </si>
+  <si>
+    <t>Timbang Inbound 7 (Bentonite)</t>
+  </si>
+  <si>
+    <t>Pemeriksaan pelumasan roll bearing 15 menit</t>
+  </si>
+  <si>
+    <t>16:00 - 17:00</t>
+  </si>
+  <si>
+    <t>Truk Outbound 5 (30 Ton)</t>
+  </si>
+  <si>
+    <t>Timbang Outbound 5</t>
+  </si>
+  <si>
+    <t>Truk tangki proyek jalan sebelum jam sibuk</t>
+  </si>
+  <si>
+    <t>17:00 - 18:00</t>
+  </si>
+  <si>
+    <t>Truk Inbound 8 (Bentonite)</t>
+  </si>
+  <si>
+    <t>Timbang Inbound 8 (Bentonite)</t>
+  </si>
+  <si>
+    <t>Level silo mendekati batas atas 60 Ton</t>
+  </si>
+  <si>
+    <t>18:00 - 19:00</t>
+  </si>
+  <si>
+    <t>Truk Outbound 6 (30 Ton)</t>
+  </si>
+  <si>
+    <t>Timbang Outbound 6</t>
+  </si>
+  <si>
+    <t>Pelepasan muatan produk jadi ke-6</t>
+  </si>
+  <si>
+    <t>19:00 - 20:00</t>
+  </si>
+  <si>
+    <t>Truk Inbound 9 (Bentonite)</t>
+  </si>
+  <si>
+    <t>Timbang Inbound 9 (Bentonite)</t>
+  </si>
+  <si>
+    <t>Antrean jembatan timbang terpantau lancar</t>
+  </si>
+  <si>
+    <t>20:00 - 21:00</t>
+  </si>
+  <si>
+    <t>Truk Outbound 7 (30 Ton)</t>
+  </si>
+  <si>
+    <t>Timbang Outbound 7</t>
+  </si>
+  <si>
+    <t>Target 210 Ton tercapai</t>
+  </si>
+  <si>
+    <t>21:00 - 22:00</t>
+  </si>
+  <si>
+    <t>Truk Inbound 10 (Calsium)</t>
+  </si>
+  <si>
+    <t>Timbang Inbound 10 (Calsium)</t>
+  </si>
+  <si>
+    <t>Waspada: Level Silo menyentuh 80 Ton!</t>
+  </si>
+  <si>
+    <t>22:00 - 23:00</t>
+  </si>
+  <si>
+    <t>Persiapan Shift 3 / Night Shift</t>
+  </si>
+  <si>
+    <t>Truk Inbound 11 (Bentonite)</t>
+  </si>
+  <si>
+    <t>Truk Outbound 8 (30 Ton)</t>
+  </si>
+  <si>
+    <t>Timbang Inbound 11 &amp; Outbound 8</t>
+  </si>
+  <si>
+    <t>Truk ke-8 berhasil dispatch, silo turun ke 70T</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="0.00&quot;%&quot;"/>
     <numFmt numFmtId="165" formatCode="&quot;Rp &quot;#,##0"/>
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
     <numFmt numFmtId="167" formatCode="#,##0.0"/>
     <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="169" formatCode="#,##0.0&quot; Ton&quot;"/>
+    <numFmt numFmtId="170" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1460,8 +2054,49 @@
       <color rgb="FF0F172A"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color rgb="FF1E293B"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.5"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.5"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="9.5"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF0F172A"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.5"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1486,8 +2121,80 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0284C7"/>
+        <bgColor rgb="FF0284C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3C7"/>
+        <bgColor rgb="FFFEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0D9488"/>
+        <bgColor rgb="FF0D9488"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCFCE7"/>
+        <bgColor rgb="FFDCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD97706"/>
+        <bgColor rgb="FFD97706"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6366F1"/>
+        <bgColor rgb="FF6366F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor rgb="FF1E293B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor rgb="FFF8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor rgb="FFDCFCE7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -1510,11 +2217,41 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF0F172A"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1E293B"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1596,6 +2333,193 @@
     </xf>
     <xf numFmtId="168" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="11" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="11" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="10" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="10" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="12" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="12" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="3" fontId="12" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2190,6 +3114,1785 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30EDEC2D-9F64-4FDF-BA12-D85301648FDD}">
+  <dimension ref="A1:R50"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="38" customWidth="1"/>
+    <col min="3" max="3" width="32" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="11" max="12" width="20" customWidth="1"/>
+    <col min="13" max="13" width="22" customWidth="1"/>
+    <col min="14" max="14" width="24" customWidth="1"/>
+    <col min="15" max="15" width="26" customWidth="1"/>
+    <col min="16" max="16" width="30" customWidth="1"/>
+    <col min="17" max="17" width="32" customWidth="1"/>
+    <col min="18" max="18" width="34" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" ht="19.8" x14ac:dyDescent="0.4">
+      <c r="A1" s="32" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A4" s="33" t="s">
+        <v>453</v>
+      </c>
+      <c r="B4" s="34"/>
+      <c r="C4" s="34"/>
+      <c r="D4" s="34"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="34"/>
+      <c r="G4" s="34"/>
+      <c r="H4" s="34"/>
+      <c r="I4" s="34"/>
+      <c r="J4" s="34"/>
+      <c r="K4" s="34"/>
+      <c r="L4" s="34"/>
+      <c r="M4" s="34"/>
+      <c r="N4" s="34"/>
+      <c r="O4" s="34"/>
+      <c r="P4" s="34"/>
+    </row>
+    <row r="5" spans="1:18" ht="28.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="35" t="s">
+        <v>454</v>
+      </c>
+      <c r="B5" s="35" t="s">
+        <v>455</v>
+      </c>
+      <c r="C5" s="35" t="s">
+        <v>456</v>
+      </c>
+      <c r="D5" s="35" t="s">
+        <v>457</v>
+      </c>
+      <c r="E5" s="35" t="s">
+        <v>458</v>
+      </c>
+      <c r="F5" s="35" t="s">
+        <v>459</v>
+      </c>
+      <c r="G5" s="35" t="s">
+        <v>460</v>
+      </c>
+      <c r="H5" s="35" t="s">
+        <v>461</v>
+      </c>
+      <c r="I5" s="35" t="s">
+        <v>462</v>
+      </c>
+      <c r="J5" s="35" t="s">
+        <v>463</v>
+      </c>
+      <c r="K5" s="35" t="s">
+        <v>464</v>
+      </c>
+      <c r="L5" s="35" t="s">
+        <v>465</v>
+      </c>
+      <c r="M5" s="35" t="s">
+        <v>466</v>
+      </c>
+      <c r="N5" s="35" t="s">
+        <v>467</v>
+      </c>
+      <c r="O5" s="35" t="s">
+        <v>468</v>
+      </c>
+      <c r="P5" s="35" t="s">
+        <v>469</v>
+      </c>
+      <c r="Q5" s="35" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="36" t="s">
+        <v>471</v>
+      </c>
+      <c r="B6" s="37" t="s">
+        <v>472</v>
+      </c>
+      <c r="C6" s="37" t="s">
+        <v>473</v>
+      </c>
+      <c r="D6" s="38">
+        <v>4</v>
+      </c>
+      <c r="E6" s="39">
+        <v>80</v>
+      </c>
+      <c r="F6" s="40">
+        <f t="shared" ref="F6:F11" si="0">E6*25</f>
+        <v>2000</v>
+      </c>
+      <c r="G6" s="41">
+        <f t="shared" ref="G6:G11" si="1">E6/30</f>
+        <v>2.6666666666666665</v>
+      </c>
+      <c r="H6" s="42">
+        <v>3</v>
+      </c>
+      <c r="I6" s="40">
+        <f t="shared" ref="I6:I11" si="2">E6*0.8</f>
+        <v>64</v>
+      </c>
+      <c r="J6" s="41">
+        <f t="shared" ref="J6:J11" si="3">I6/30</f>
+        <v>2.1333333333333333</v>
+      </c>
+      <c r="K6" s="40">
+        <f t="shared" ref="K6:K11" si="4">E6*0.15</f>
+        <v>12</v>
+      </c>
+      <c r="L6" s="40">
+        <f t="shared" ref="L6:L11" si="5">E6*0.05</f>
+        <v>4</v>
+      </c>
+      <c r="M6" s="42">
+        <v>3</v>
+      </c>
+      <c r="N6" s="42">
+        <f t="shared" ref="N6:N11" si="6">H6+M6</f>
+        <v>6</v>
+      </c>
+      <c r="O6" s="41">
+        <f t="shared" ref="O6:O11" si="7">134.4/(I6/D6)</f>
+        <v>8.4</v>
+      </c>
+      <c r="P6" s="41">
+        <f t="shared" ref="P6:P11" si="8">86.4/(E6/D6)</f>
+        <v>4.32</v>
+      </c>
+      <c r="Q6" s="37" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="43" t="s">
+        <v>475</v>
+      </c>
+      <c r="B7" s="44" t="s">
+        <v>476</v>
+      </c>
+      <c r="C7" s="44" t="s">
+        <v>477</v>
+      </c>
+      <c r="D7" s="45">
+        <v>7</v>
+      </c>
+      <c r="E7" s="46">
+        <v>140</v>
+      </c>
+      <c r="F7" s="47">
+        <f t="shared" si="0"/>
+        <v>3500</v>
+      </c>
+      <c r="G7" s="48">
+        <f t="shared" si="1"/>
+        <v>4.666666666666667</v>
+      </c>
+      <c r="H7" s="49">
+        <v>5</v>
+      </c>
+      <c r="I7" s="47">
+        <f t="shared" si="2"/>
+        <v>112</v>
+      </c>
+      <c r="J7" s="48">
+        <f t="shared" si="3"/>
+        <v>3.7333333333333334</v>
+      </c>
+      <c r="K7" s="47">
+        <f t="shared" si="4"/>
+        <v>21</v>
+      </c>
+      <c r="L7" s="47">
+        <f t="shared" si="5"/>
+        <v>7</v>
+      </c>
+      <c r="M7" s="49">
+        <v>5</v>
+      </c>
+      <c r="N7" s="49">
+        <f t="shared" si="6"/>
+        <v>10</v>
+      </c>
+      <c r="O7" s="48">
+        <f t="shared" si="7"/>
+        <v>8.4</v>
+      </c>
+      <c r="P7" s="48">
+        <f t="shared" si="8"/>
+        <v>4.32</v>
+      </c>
+      <c r="Q7" s="44" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="36" t="s">
+        <v>479</v>
+      </c>
+      <c r="B8" s="37" t="s">
+        <v>480</v>
+      </c>
+      <c r="C8" s="37" t="s">
+        <v>481</v>
+      </c>
+      <c r="D8" s="38">
+        <v>10</v>
+      </c>
+      <c r="E8" s="39">
+        <v>200</v>
+      </c>
+      <c r="F8" s="40">
+        <f t="shared" si="0"/>
+        <v>5000</v>
+      </c>
+      <c r="G8" s="41">
+        <f t="shared" si="1"/>
+        <v>6.666666666666667</v>
+      </c>
+      <c r="H8" s="42">
+        <v>7</v>
+      </c>
+      <c r="I8" s="40">
+        <f t="shared" si="2"/>
+        <v>160</v>
+      </c>
+      <c r="J8" s="41">
+        <f t="shared" si="3"/>
+        <v>5.333333333333333</v>
+      </c>
+      <c r="K8" s="40">
+        <f t="shared" si="4"/>
+        <v>30</v>
+      </c>
+      <c r="L8" s="40">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M8" s="42">
+        <v>7</v>
+      </c>
+      <c r="N8" s="42">
+        <f t="shared" si="6"/>
+        <v>14</v>
+      </c>
+      <c r="O8" s="41">
+        <f t="shared" si="7"/>
+        <v>8.4</v>
+      </c>
+      <c r="P8" s="41">
+        <f t="shared" si="8"/>
+        <v>4.32</v>
+      </c>
+      <c r="Q8" s="37" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="43" t="s">
+        <v>483</v>
+      </c>
+      <c r="B9" s="44" t="s">
+        <v>484</v>
+      </c>
+      <c r="C9" s="44" t="s">
+        <v>485</v>
+      </c>
+      <c r="D9" s="45">
+        <v>14</v>
+      </c>
+      <c r="E9" s="46">
+        <v>280</v>
+      </c>
+      <c r="F9" s="47">
+        <f t="shared" si="0"/>
+        <v>7000</v>
+      </c>
+      <c r="G9" s="48">
+        <f t="shared" si="1"/>
+        <v>9.3333333333333339</v>
+      </c>
+      <c r="H9" s="49">
+        <v>10</v>
+      </c>
+      <c r="I9" s="47">
+        <f t="shared" si="2"/>
+        <v>224</v>
+      </c>
+      <c r="J9" s="48">
+        <f t="shared" si="3"/>
+        <v>7.4666666666666668</v>
+      </c>
+      <c r="K9" s="47">
+        <f t="shared" si="4"/>
+        <v>42</v>
+      </c>
+      <c r="L9" s="47">
+        <f t="shared" si="5"/>
+        <v>14</v>
+      </c>
+      <c r="M9" s="49">
+        <v>10</v>
+      </c>
+      <c r="N9" s="49">
+        <f t="shared" si="6"/>
+        <v>20</v>
+      </c>
+      <c r="O9" s="48">
+        <f t="shared" si="7"/>
+        <v>8.4</v>
+      </c>
+      <c r="P9" s="48">
+        <f t="shared" si="8"/>
+        <v>4.32</v>
+      </c>
+      <c r="Q9" s="44" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="36" t="s">
+        <v>487</v>
+      </c>
+      <c r="B10" s="37" t="s">
+        <v>488</v>
+      </c>
+      <c r="C10" s="37" t="s">
+        <v>489</v>
+      </c>
+      <c r="D10" s="38">
+        <v>18</v>
+      </c>
+      <c r="E10" s="39">
+        <v>360</v>
+      </c>
+      <c r="F10" s="40">
+        <f t="shared" si="0"/>
+        <v>9000</v>
+      </c>
+      <c r="G10" s="41">
+        <f t="shared" si="1"/>
+        <v>12</v>
+      </c>
+      <c r="H10" s="42">
+        <v>12</v>
+      </c>
+      <c r="I10" s="40">
+        <f t="shared" si="2"/>
+        <v>288</v>
+      </c>
+      <c r="J10" s="41">
+        <f t="shared" si="3"/>
+        <v>9.6</v>
+      </c>
+      <c r="K10" s="40">
+        <f t="shared" si="4"/>
+        <v>54</v>
+      </c>
+      <c r="L10" s="40">
+        <f t="shared" si="5"/>
+        <v>18</v>
+      </c>
+      <c r="M10" s="42">
+        <v>13</v>
+      </c>
+      <c r="N10" s="42">
+        <f t="shared" si="6"/>
+        <v>25</v>
+      </c>
+      <c r="O10" s="41">
+        <f t="shared" si="7"/>
+        <v>8.4</v>
+      </c>
+      <c r="P10" s="41">
+        <f t="shared" si="8"/>
+        <v>4.32</v>
+      </c>
+      <c r="Q10" s="37" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="50" t="s">
+        <v>491</v>
+      </c>
+      <c r="B11" s="51" t="s">
+        <v>492</v>
+      </c>
+      <c r="C11" s="51" t="s">
+        <v>493</v>
+      </c>
+      <c r="D11" s="52">
+        <v>21</v>
+      </c>
+      <c r="E11" s="53">
+        <v>420</v>
+      </c>
+      <c r="F11" s="54">
+        <f t="shared" si="0"/>
+        <v>10500</v>
+      </c>
+      <c r="G11" s="55">
+        <f t="shared" si="1"/>
+        <v>14</v>
+      </c>
+      <c r="H11" s="56">
+        <v>14</v>
+      </c>
+      <c r="I11" s="54">
+        <f t="shared" si="2"/>
+        <v>336</v>
+      </c>
+      <c r="J11" s="55">
+        <f t="shared" si="3"/>
+        <v>11.2</v>
+      </c>
+      <c r="K11" s="54">
+        <f t="shared" si="4"/>
+        <v>63</v>
+      </c>
+      <c r="L11" s="54">
+        <f t="shared" si="5"/>
+        <v>21</v>
+      </c>
+      <c r="M11" s="56">
+        <v>15</v>
+      </c>
+      <c r="N11" s="56">
+        <f t="shared" si="6"/>
+        <v>29</v>
+      </c>
+      <c r="O11" s="55">
+        <f t="shared" si="7"/>
+        <v>8.4</v>
+      </c>
+      <c r="P11" s="55">
+        <f t="shared" si="8"/>
+        <v>4.32</v>
+      </c>
+      <c r="Q11" s="51" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A12" s="57"/>
+      <c r="B12" s="58"/>
+      <c r="C12" s="58"/>
+      <c r="D12" s="58"/>
+      <c r="E12" s="58"/>
+      <c r="F12" s="58"/>
+      <c r="G12" s="58"/>
+      <c r="H12" s="58"/>
+      <c r="I12" s="58"/>
+      <c r="J12" s="58"/>
+      <c r="K12" s="58"/>
+      <c r="L12" s="58"/>
+      <c r="M12" s="58"/>
+      <c r="N12" s="58"/>
+      <c r="O12" s="58"/>
+      <c r="P12" s="58"/>
+    </row>
+    <row r="13" spans="1:18" ht="28.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="59" t="s">
+        <v>495</v>
+      </c>
+      <c r="B13" s="60"/>
+      <c r="C13" s="60"/>
+      <c r="D13" s="60"/>
+      <c r="E13" s="60"/>
+      <c r="F13" s="60"/>
+      <c r="G13" s="60"/>
+      <c r="H13" s="60"/>
+      <c r="I13" s="60"/>
+      <c r="J13" s="60"/>
+      <c r="K13" s="60"/>
+      <c r="L13" s="60"/>
+      <c r="M13" s="60"/>
+      <c r="N13" s="60"/>
+      <c r="O13" s="60"/>
+      <c r="P13" s="89"/>
+      <c r="Q13" s="90"/>
+      <c r="R13" s="90"/>
+    </row>
+    <row r="14" spans="1:18" ht="22.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="35" t="s">
+        <v>454</v>
+      </c>
+      <c r="B14" s="61" t="s">
+        <v>496</v>
+      </c>
+      <c r="C14" s="62" t="s">
+        <v>497</v>
+      </c>
+      <c r="D14" s="62" t="s">
+        <v>498</v>
+      </c>
+      <c r="E14" s="62" t="s">
+        <v>499</v>
+      </c>
+      <c r="F14" s="62" t="s">
+        <v>500</v>
+      </c>
+      <c r="G14" s="62" t="s">
+        <v>501</v>
+      </c>
+      <c r="H14" s="62" t="s">
+        <v>502</v>
+      </c>
+      <c r="I14" s="62" t="s">
+        <v>503</v>
+      </c>
+      <c r="J14" s="62" t="s">
+        <v>504</v>
+      </c>
+      <c r="K14" s="62" t="s">
+        <v>505</v>
+      </c>
+      <c r="L14" s="62" t="s">
+        <v>506</v>
+      </c>
+      <c r="M14" s="62" t="s">
+        <v>507</v>
+      </c>
+      <c r="N14" s="63" t="s">
+        <v>508</v>
+      </c>
+      <c r="O14" s="62" t="s">
+        <v>509</v>
+      </c>
+      <c r="P14" s="97" t="s">
+        <v>510</v>
+      </c>
+      <c r="Q14" s="98" t="s">
+        <v>511</v>
+      </c>
+      <c r="R14" s="98" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="43" t="s">
+        <v>471</v>
+      </c>
+      <c r="B15" s="47">
+        <f t="shared" ref="B15:B20" si="9">E6</f>
+        <v>80</v>
+      </c>
+      <c r="C15" s="64">
+        <f t="shared" ref="C15:C20" si="10">B15*3582500</f>
+        <v>286600000</v>
+      </c>
+      <c r="D15" s="64">
+        <f t="shared" ref="D15:D20" si="11">B15*79930</f>
+        <v>6394400</v>
+      </c>
+      <c r="E15" s="64">
+        <f t="shared" ref="E15:E20" si="12">B15*7223</f>
+        <v>577840</v>
+      </c>
+      <c r="F15" s="64">
+        <f t="shared" ref="F15:F20" si="13">B15*4738</f>
+        <v>379040</v>
+      </c>
+      <c r="G15" s="64">
+        <v>2675000</v>
+      </c>
+      <c r="H15" s="64">
+        <f t="shared" ref="H15:H20" si="14">B15*139006</f>
+        <v>11120480</v>
+      </c>
+      <c r="I15" s="65">
+        <f t="shared" ref="I15:I20" si="15">SUM(C15:H15)</f>
+        <v>307746760</v>
+      </c>
+      <c r="J15" s="64">
+        <f t="shared" ref="J15:J20" si="16">I15/B15</f>
+        <v>3846834.5</v>
+      </c>
+      <c r="K15" s="64">
+        <v>4350000</v>
+      </c>
+      <c r="L15" s="65">
+        <f t="shared" ref="L15:L20" si="17">B15*K15</f>
+        <v>348000000</v>
+      </c>
+      <c r="M15" s="65">
+        <f t="shared" ref="M15:M20" si="18">L15-I15</f>
+        <v>40253240</v>
+      </c>
+      <c r="N15" s="66">
+        <f t="shared" ref="N15:N20" si="19">M15/L15</f>
+        <v>0.11567022988505747</v>
+      </c>
+      <c r="O15" s="64">
+        <f t="shared" ref="O15:O20" si="20">M15*25</f>
+        <v>1006331000</v>
+      </c>
+      <c r="P15" s="91">
+        <f t="shared" ref="P15:P20" si="21">I15*30</f>
+        <v>9232402800</v>
+      </c>
+      <c r="Q15" s="91">
+        <f t="shared" ref="Q15:Q20" si="22">I15*60</f>
+        <v>18464805600</v>
+      </c>
+      <c r="R15" s="92">
+        <f t="shared" ref="R15:R20" si="23">I15*90</f>
+        <v>27697208400</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="36" t="s">
+        <v>475</v>
+      </c>
+      <c r="B16" s="40">
+        <f t="shared" si="9"/>
+        <v>140</v>
+      </c>
+      <c r="C16" s="67">
+        <f t="shared" si="10"/>
+        <v>501550000</v>
+      </c>
+      <c r="D16" s="67">
+        <f t="shared" si="11"/>
+        <v>11190200</v>
+      </c>
+      <c r="E16" s="67">
+        <f t="shared" si="12"/>
+        <v>1011220</v>
+      </c>
+      <c r="F16" s="67">
+        <f t="shared" si="13"/>
+        <v>663320</v>
+      </c>
+      <c r="G16" s="67">
+        <v>2675000</v>
+      </c>
+      <c r="H16" s="67">
+        <f t="shared" si="14"/>
+        <v>19460840</v>
+      </c>
+      <c r="I16" s="68">
+        <f t="shared" si="15"/>
+        <v>536550580</v>
+      </c>
+      <c r="J16" s="67">
+        <f t="shared" si="16"/>
+        <v>3832504.1428571427</v>
+      </c>
+      <c r="K16" s="67">
+        <v>4350000</v>
+      </c>
+      <c r="L16" s="68">
+        <f t="shared" si="17"/>
+        <v>609000000</v>
+      </c>
+      <c r="M16" s="68">
+        <f t="shared" si="18"/>
+        <v>72449420</v>
+      </c>
+      <c r="N16" s="69">
+        <f t="shared" si="19"/>
+        <v>0.11896456486042693</v>
+      </c>
+      <c r="O16" s="67">
+        <f t="shared" si="20"/>
+        <v>1811235500</v>
+      </c>
+      <c r="P16" s="93">
+        <f t="shared" si="21"/>
+        <v>16096517400</v>
+      </c>
+      <c r="Q16" s="93">
+        <f t="shared" si="22"/>
+        <v>32193034800</v>
+      </c>
+      <c r="R16" s="94">
+        <f t="shared" si="23"/>
+        <v>48289552200</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="43" t="s">
+        <v>479</v>
+      </c>
+      <c r="B17" s="47">
+        <f t="shared" si="9"/>
+        <v>200</v>
+      </c>
+      <c r="C17" s="64">
+        <f t="shared" si="10"/>
+        <v>716500000</v>
+      </c>
+      <c r="D17" s="64">
+        <f t="shared" si="11"/>
+        <v>15986000</v>
+      </c>
+      <c r="E17" s="64">
+        <f t="shared" si="12"/>
+        <v>1444600</v>
+      </c>
+      <c r="F17" s="64">
+        <f t="shared" si="13"/>
+        <v>947600</v>
+      </c>
+      <c r="G17" s="64">
+        <v>4776785</v>
+      </c>
+      <c r="H17" s="64">
+        <f t="shared" si="14"/>
+        <v>27801200</v>
+      </c>
+      <c r="I17" s="65">
+        <f t="shared" si="15"/>
+        <v>767456185</v>
+      </c>
+      <c r="J17" s="64">
+        <f t="shared" si="16"/>
+        <v>3837280.9249999998</v>
+      </c>
+      <c r="K17" s="64">
+        <v>4350000</v>
+      </c>
+      <c r="L17" s="65">
+        <f t="shared" si="17"/>
+        <v>870000000</v>
+      </c>
+      <c r="M17" s="65">
+        <f t="shared" si="18"/>
+        <v>102543815</v>
+      </c>
+      <c r="N17" s="66">
+        <f t="shared" si="19"/>
+        <v>0.11786645402298851</v>
+      </c>
+      <c r="O17" s="64">
+        <f t="shared" si="20"/>
+        <v>2563595375</v>
+      </c>
+      <c r="P17" s="91">
+        <f t="shared" si="21"/>
+        <v>23023685550</v>
+      </c>
+      <c r="Q17" s="91">
+        <f t="shared" si="22"/>
+        <v>46047371100</v>
+      </c>
+      <c r="R17" s="92">
+        <f t="shared" si="23"/>
+        <v>69071056650</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="84" t="s">
+        <v>483</v>
+      </c>
+      <c r="B18" s="85">
+        <f t="shared" si="9"/>
+        <v>280</v>
+      </c>
+      <c r="C18" s="86">
+        <f t="shared" si="10"/>
+        <v>1003100000</v>
+      </c>
+      <c r="D18" s="86">
+        <f t="shared" si="11"/>
+        <v>22380400</v>
+      </c>
+      <c r="E18" s="86">
+        <f t="shared" si="12"/>
+        <v>2022440</v>
+      </c>
+      <c r="F18" s="86">
+        <f t="shared" si="13"/>
+        <v>1326640</v>
+      </c>
+      <c r="G18" s="86">
+        <v>5617500</v>
+      </c>
+      <c r="H18" s="86">
+        <f t="shared" si="14"/>
+        <v>38921680</v>
+      </c>
+      <c r="I18" s="87">
+        <f t="shared" si="15"/>
+        <v>1073368660</v>
+      </c>
+      <c r="J18" s="86">
+        <f t="shared" si="16"/>
+        <v>3833459.5</v>
+      </c>
+      <c r="K18" s="86">
+        <v>4350000</v>
+      </c>
+      <c r="L18" s="87">
+        <f t="shared" si="17"/>
+        <v>1218000000</v>
+      </c>
+      <c r="M18" s="87">
+        <f t="shared" si="18"/>
+        <v>144631340</v>
+      </c>
+      <c r="N18" s="88">
+        <f t="shared" si="19"/>
+        <v>0.11874494252873563</v>
+      </c>
+      <c r="O18" s="86">
+        <f t="shared" si="20"/>
+        <v>3615783500</v>
+      </c>
+      <c r="P18" s="93">
+        <f t="shared" si="21"/>
+        <v>32201059800</v>
+      </c>
+      <c r="Q18" s="93">
+        <f t="shared" si="22"/>
+        <v>64402119600</v>
+      </c>
+      <c r="R18" s="94">
+        <f t="shared" si="23"/>
+        <v>96603179400</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A19" s="43" t="s">
+        <v>487</v>
+      </c>
+      <c r="B19" s="47">
+        <f t="shared" si="9"/>
+        <v>360</v>
+      </c>
+      <c r="C19" s="64">
+        <f t="shared" si="10"/>
+        <v>1289700000</v>
+      </c>
+      <c r="D19" s="64">
+        <f t="shared" si="11"/>
+        <v>28774800</v>
+      </c>
+      <c r="E19" s="64">
+        <f t="shared" si="12"/>
+        <v>2600280</v>
+      </c>
+      <c r="F19" s="64">
+        <f t="shared" si="13"/>
+        <v>1705680</v>
+      </c>
+      <c r="G19" s="64">
+        <v>7720000</v>
+      </c>
+      <c r="H19" s="64">
+        <f t="shared" si="14"/>
+        <v>50042160</v>
+      </c>
+      <c r="I19" s="65">
+        <f t="shared" si="15"/>
+        <v>1380542920</v>
+      </c>
+      <c r="J19" s="64">
+        <f t="shared" si="16"/>
+        <v>3834841.4444444445</v>
+      </c>
+      <c r="K19" s="64">
+        <v>4350000</v>
+      </c>
+      <c r="L19" s="65">
+        <f t="shared" si="17"/>
+        <v>1566000000</v>
+      </c>
+      <c r="M19" s="65">
+        <f t="shared" si="18"/>
+        <v>185457080</v>
+      </c>
+      <c r="N19" s="66">
+        <f t="shared" si="19"/>
+        <v>0.11842725415070243</v>
+      </c>
+      <c r="O19" s="64">
+        <f t="shared" si="20"/>
+        <v>4636427000</v>
+      </c>
+      <c r="P19" s="91">
+        <f t="shared" si="21"/>
+        <v>41416287600</v>
+      </c>
+      <c r="Q19" s="91">
+        <f t="shared" si="22"/>
+        <v>82832575200</v>
+      </c>
+      <c r="R19" s="92">
+        <f t="shared" si="23"/>
+        <v>124248862800</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A20" s="70" t="s">
+        <v>491</v>
+      </c>
+      <c r="B20" s="71">
+        <f t="shared" si="9"/>
+        <v>420</v>
+      </c>
+      <c r="C20" s="72">
+        <f t="shared" si="10"/>
+        <v>1504650000</v>
+      </c>
+      <c r="D20" s="72">
+        <f t="shared" si="11"/>
+        <v>33570600</v>
+      </c>
+      <c r="E20" s="72">
+        <f t="shared" si="12"/>
+        <v>3033660</v>
+      </c>
+      <c r="F20" s="72">
+        <f t="shared" si="13"/>
+        <v>1989960</v>
+      </c>
+      <c r="G20" s="72">
+        <v>9844000</v>
+      </c>
+      <c r="H20" s="72">
+        <f t="shared" si="14"/>
+        <v>58382520</v>
+      </c>
+      <c r="I20" s="73">
+        <f t="shared" si="15"/>
+        <v>1611470740</v>
+      </c>
+      <c r="J20" s="72">
+        <f t="shared" si="16"/>
+        <v>3836835.0952380951</v>
+      </c>
+      <c r="K20" s="72">
+        <v>4350000</v>
+      </c>
+      <c r="L20" s="73">
+        <f t="shared" si="17"/>
+        <v>1827000000</v>
+      </c>
+      <c r="M20" s="73">
+        <f t="shared" si="18"/>
+        <v>215529260</v>
+      </c>
+      <c r="N20" s="74">
+        <f t="shared" si="19"/>
+        <v>0.11796894362342639</v>
+      </c>
+      <c r="O20" s="72">
+        <f t="shared" si="20"/>
+        <v>5388231500</v>
+      </c>
+      <c r="P20" s="95">
+        <f t="shared" si="21"/>
+        <v>48344122200</v>
+      </c>
+      <c r="Q20" s="95">
+        <f t="shared" si="22"/>
+        <v>96688244400</v>
+      </c>
+      <c r="R20" s="96">
+        <f t="shared" si="23"/>
+        <v>145032366600</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" ht="25.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="60"/>
+      <c r="B21" s="60"/>
+      <c r="C21" s="60"/>
+      <c r="D21" s="60"/>
+      <c r="E21" s="60"/>
+      <c r="F21" s="60"/>
+      <c r="G21" s="60"/>
+    </row>
+    <row r="22" spans="1:18" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="75" t="s">
+        <v>513</v>
+      </c>
+      <c r="B22" s="76"/>
+      <c r="C22" s="77"/>
+      <c r="D22" s="77"/>
+      <c r="E22" s="76"/>
+      <c r="F22" s="78"/>
+      <c r="G22" s="77"/>
+    </row>
+    <row r="23" spans="1:18" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="35" t="s">
+        <v>2</v>
+      </c>
+      <c r="B23" s="35" t="s">
+        <v>514</v>
+      </c>
+      <c r="C23" s="35" t="s">
+        <v>515</v>
+      </c>
+      <c r="D23" s="35" t="s">
+        <v>516</v>
+      </c>
+      <c r="E23" s="35" t="s">
+        <v>517</v>
+      </c>
+      <c r="F23" s="35" t="s">
+        <v>518</v>
+      </c>
+      <c r="G23" s="35" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="36">
+        <v>1</v>
+      </c>
+      <c r="B24" s="79" t="s">
+        <v>520</v>
+      </c>
+      <c r="C24" s="37" t="s">
+        <v>521</v>
+      </c>
+      <c r="D24" s="37" t="s">
+        <v>522</v>
+      </c>
+      <c r="E24" s="37" t="s">
+        <v>523</v>
+      </c>
+      <c r="F24" s="80" t="s">
+        <v>524</v>
+      </c>
+      <c r="G24" s="37" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="43">
+        <v>2</v>
+      </c>
+      <c r="B25" s="81" t="s">
+        <v>526</v>
+      </c>
+      <c r="C25" s="44" t="s">
+        <v>527</v>
+      </c>
+      <c r="D25" s="44" t="s">
+        <v>528</v>
+      </c>
+      <c r="E25" s="44" t="s">
+        <v>529</v>
+      </c>
+      <c r="F25" s="82" t="s">
+        <v>530</v>
+      </c>
+      <c r="G25" s="44" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="36">
+        <v>3</v>
+      </c>
+      <c r="B26" s="79" t="s">
+        <v>532</v>
+      </c>
+      <c r="C26" s="37" t="s">
+        <v>533</v>
+      </c>
+      <c r="D26" s="37" t="s">
+        <v>534</v>
+      </c>
+      <c r="E26" s="37" t="s">
+        <v>535</v>
+      </c>
+      <c r="F26" s="80" t="s">
+        <v>536</v>
+      </c>
+      <c r="G26" s="37" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="43">
+        <v>4</v>
+      </c>
+      <c r="B27" s="81" t="s">
+        <v>538</v>
+      </c>
+      <c r="C27" s="44" t="s">
+        <v>539</v>
+      </c>
+      <c r="D27" s="44" t="s">
+        <v>540</v>
+      </c>
+      <c r="E27" s="44" t="s">
+        <v>541</v>
+      </c>
+      <c r="F27" s="82" t="s">
+        <v>530</v>
+      </c>
+      <c r="G27" s="44" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="36">
+        <v>5</v>
+      </c>
+      <c r="B28" s="79" t="s">
+        <v>543</v>
+      </c>
+      <c r="C28" s="37" t="s">
+        <v>544</v>
+      </c>
+      <c r="D28" s="37" t="s">
+        <v>545</v>
+      </c>
+      <c r="E28" s="37" t="s">
+        <v>546</v>
+      </c>
+      <c r="F28" s="80" t="s">
+        <v>530</v>
+      </c>
+      <c r="G28" s="37" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" ht="88.2" x14ac:dyDescent="0.3">
+      <c r="A29" s="43">
+        <v>6</v>
+      </c>
+      <c r="B29" s="81" t="s">
+        <v>548</v>
+      </c>
+      <c r="C29" s="44" t="s">
+        <v>549</v>
+      </c>
+      <c r="D29" s="44" t="s">
+        <v>550</v>
+      </c>
+      <c r="E29" s="44" t="s">
+        <v>551</v>
+      </c>
+      <c r="F29" s="82" t="s">
+        <v>524</v>
+      </c>
+      <c r="G29" s="44" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" ht="75.599999999999994" x14ac:dyDescent="0.3">
+      <c r="A30" s="36">
+        <v>7</v>
+      </c>
+      <c r="B30" s="79" t="s">
+        <v>553</v>
+      </c>
+      <c r="C30" s="37" t="s">
+        <v>554</v>
+      </c>
+      <c r="D30" s="37" t="s">
+        <v>555</v>
+      </c>
+      <c r="E30" s="37" t="s">
+        <v>556</v>
+      </c>
+      <c r="F30" s="80" t="s">
+        <v>557</v>
+      </c>
+      <c r="G30" s="37" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" ht="75.599999999999994" x14ac:dyDescent="0.3">
+      <c r="A31" s="43">
+        <v>8</v>
+      </c>
+      <c r="B31" s="81" t="s">
+        <v>559</v>
+      </c>
+      <c r="C31" s="44" t="s">
+        <v>560</v>
+      </c>
+      <c r="D31" s="44" t="s">
+        <v>561</v>
+      </c>
+      <c r="E31" s="44" t="s">
+        <v>562</v>
+      </c>
+      <c r="F31" s="82" t="s">
+        <v>530</v>
+      </c>
+      <c r="G31" s="44" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A33" s="83" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="25.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="35" t="s">
+        <v>565</v>
+      </c>
+      <c r="B34" s="35" t="s">
+        <v>566</v>
+      </c>
+      <c r="C34" s="35" t="s">
+        <v>567</v>
+      </c>
+      <c r="D34" s="35" t="s">
+        <v>568</v>
+      </c>
+      <c r="E34" s="35" t="s">
+        <v>569</v>
+      </c>
+      <c r="F34" s="35" t="s">
+        <v>570</v>
+      </c>
+      <c r="G34" s="35" t="s">
+        <v>571</v>
+      </c>
+      <c r="H34" s="35" t="s">
+        <v>572</v>
+      </c>
+      <c r="I34" s="35" t="s">
+        <v>573</v>
+      </c>
+      <c r="J34" s="35" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A35" s="43" t="s">
+        <v>575</v>
+      </c>
+      <c r="B35" s="44" t="s">
+        <v>576</v>
+      </c>
+      <c r="C35" s="44" t="s">
+        <v>577</v>
+      </c>
+      <c r="D35" s="44" t="s">
+        <v>578</v>
+      </c>
+      <c r="E35" s="46">
+        <v>30</v>
+      </c>
+      <c r="F35" s="46">
+        <v>0</v>
+      </c>
+      <c r="G35" s="47">
+        <v>114.4</v>
+      </c>
+      <c r="H35" s="46">
+        <v>30</v>
+      </c>
+      <c r="I35" s="44" t="s">
+        <v>579</v>
+      </c>
+      <c r="J35" s="44" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A36" s="36" t="s">
+        <v>581</v>
+      </c>
+      <c r="B36" s="37" t="s">
+        <v>582</v>
+      </c>
+      <c r="C36" s="37" t="s">
+        <v>583</v>
+      </c>
+      <c r="D36" s="37" t="s">
+        <v>584</v>
+      </c>
+      <c r="E36" s="39">
+        <v>30</v>
+      </c>
+      <c r="F36" s="39">
+        <v>30</v>
+      </c>
+      <c r="G36" s="40">
+        <v>128.4</v>
+      </c>
+      <c r="H36" s="39">
+        <v>20</v>
+      </c>
+      <c r="I36" s="37" t="s">
+        <v>585</v>
+      </c>
+      <c r="J36" s="37" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A37" s="43" t="s">
+        <v>587</v>
+      </c>
+      <c r="B37" s="44" t="s">
+        <v>582</v>
+      </c>
+      <c r="C37" s="44" t="s">
+        <v>588</v>
+      </c>
+      <c r="D37" s="44" t="s">
+        <v>578</v>
+      </c>
+      <c r="E37" s="46">
+        <v>30</v>
+      </c>
+      <c r="F37" s="46">
+        <v>0</v>
+      </c>
+      <c r="G37" s="47">
+        <v>112.4</v>
+      </c>
+      <c r="H37" s="46">
+        <v>40</v>
+      </c>
+      <c r="I37" s="44" t="s">
+        <v>589</v>
+      </c>
+      <c r="J37" s="44" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A38" s="36" t="s">
+        <v>591</v>
+      </c>
+      <c r="B38" s="37" t="s">
+        <v>582</v>
+      </c>
+      <c r="C38" s="37" t="s">
+        <v>592</v>
+      </c>
+      <c r="D38" s="37" t="s">
+        <v>593</v>
+      </c>
+      <c r="E38" s="39">
+        <v>30</v>
+      </c>
+      <c r="F38" s="39">
+        <v>30</v>
+      </c>
+      <c r="G38" s="40">
+        <v>126.4</v>
+      </c>
+      <c r="H38" s="39">
+        <v>30</v>
+      </c>
+      <c r="I38" s="37" t="s">
+        <v>594</v>
+      </c>
+      <c r="J38" s="37" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A39" s="43" t="s">
+        <v>596</v>
+      </c>
+      <c r="B39" s="44" t="s">
+        <v>582</v>
+      </c>
+      <c r="C39" s="44" t="s">
+        <v>597</v>
+      </c>
+      <c r="D39" s="44" t="s">
+        <v>578</v>
+      </c>
+      <c r="E39" s="46">
+        <v>20</v>
+      </c>
+      <c r="F39" s="46">
+        <v>0</v>
+      </c>
+      <c r="G39" s="47">
+        <v>110.4</v>
+      </c>
+      <c r="H39" s="46">
+        <v>50</v>
+      </c>
+      <c r="I39" s="44" t="s">
+        <v>598</v>
+      </c>
+      <c r="J39" s="44" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A40" s="36" t="s">
+        <v>600</v>
+      </c>
+      <c r="B40" s="37" t="s">
+        <v>601</v>
+      </c>
+      <c r="C40" s="37" t="s">
+        <v>578</v>
+      </c>
+      <c r="D40" s="37" t="s">
+        <v>602</v>
+      </c>
+      <c r="E40" s="39">
+        <v>0</v>
+      </c>
+      <c r="F40" s="39">
+        <v>30</v>
+      </c>
+      <c r="G40" s="40">
+        <v>110.4</v>
+      </c>
+      <c r="H40" s="39">
+        <v>20</v>
+      </c>
+      <c r="I40" s="37" t="s">
+        <v>603</v>
+      </c>
+      <c r="J40" s="37" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A41" s="43" t="s">
+        <v>605</v>
+      </c>
+      <c r="B41" s="44" t="s">
+        <v>582</v>
+      </c>
+      <c r="C41" s="44" t="s">
+        <v>606</v>
+      </c>
+      <c r="D41" s="44" t="s">
+        <v>578</v>
+      </c>
+      <c r="E41" s="46">
+        <v>30</v>
+      </c>
+      <c r="F41" s="46">
+        <v>0</v>
+      </c>
+      <c r="G41" s="47">
+        <v>124.4</v>
+      </c>
+      <c r="H41" s="46">
+        <v>40</v>
+      </c>
+      <c r="I41" s="44" t="s">
+        <v>607</v>
+      </c>
+      <c r="J41" s="44" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A42" s="36" t="s">
+        <v>609</v>
+      </c>
+      <c r="B42" s="37" t="s">
+        <v>582</v>
+      </c>
+      <c r="C42" s="37" t="s">
+        <v>578</v>
+      </c>
+      <c r="D42" s="37" t="s">
+        <v>610</v>
+      </c>
+      <c r="E42" s="39">
+        <v>0</v>
+      </c>
+      <c r="F42" s="39">
+        <v>30</v>
+      </c>
+      <c r="G42" s="40">
+        <v>108.4</v>
+      </c>
+      <c r="H42" s="39">
+        <v>30</v>
+      </c>
+      <c r="I42" s="37" t="s">
+        <v>611</v>
+      </c>
+      <c r="J42" s="37" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A43" s="43" t="s">
+        <v>613</v>
+      </c>
+      <c r="B43" s="44" t="s">
+        <v>614</v>
+      </c>
+      <c r="C43" s="44" t="s">
+        <v>615</v>
+      </c>
+      <c r="D43" s="44" t="s">
+        <v>578</v>
+      </c>
+      <c r="E43" s="46">
+        <v>30</v>
+      </c>
+      <c r="F43" s="46">
+        <v>0</v>
+      </c>
+      <c r="G43" s="47">
+        <v>122.4</v>
+      </c>
+      <c r="H43" s="46">
+        <v>50</v>
+      </c>
+      <c r="I43" s="44" t="s">
+        <v>616</v>
+      </c>
+      <c r="J43" s="44" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A44" s="36" t="s">
+        <v>618</v>
+      </c>
+      <c r="B44" s="37" t="s">
+        <v>582</v>
+      </c>
+      <c r="C44" s="37" t="s">
+        <v>578</v>
+      </c>
+      <c r="D44" s="37" t="s">
+        <v>619</v>
+      </c>
+      <c r="E44" s="39">
+        <v>0</v>
+      </c>
+      <c r="F44" s="39">
+        <v>30</v>
+      </c>
+      <c r="G44" s="40">
+        <v>106.4</v>
+      </c>
+      <c r="H44" s="39">
+        <v>40</v>
+      </c>
+      <c r="I44" s="37" t="s">
+        <v>620</v>
+      </c>
+      <c r="J44" s="37" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A45" s="43" t="s">
+        <v>622</v>
+      </c>
+      <c r="B45" s="44" t="s">
+        <v>582</v>
+      </c>
+      <c r="C45" s="44" t="s">
+        <v>623</v>
+      </c>
+      <c r="D45" s="44" t="s">
+        <v>578</v>
+      </c>
+      <c r="E45" s="46">
+        <v>30</v>
+      </c>
+      <c r="F45" s="46">
+        <v>0</v>
+      </c>
+      <c r="G45" s="47">
+        <v>120.4</v>
+      </c>
+      <c r="H45" s="46">
+        <v>60</v>
+      </c>
+      <c r="I45" s="44" t="s">
+        <v>624</v>
+      </c>
+      <c r="J45" s="44" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A46" s="36" t="s">
+        <v>626</v>
+      </c>
+      <c r="B46" s="37" t="s">
+        <v>582</v>
+      </c>
+      <c r="C46" s="37" t="s">
+        <v>578</v>
+      </c>
+      <c r="D46" s="37" t="s">
+        <v>627</v>
+      </c>
+      <c r="E46" s="39">
+        <v>0</v>
+      </c>
+      <c r="F46" s="39">
+        <v>30</v>
+      </c>
+      <c r="G46" s="40">
+        <v>104.4</v>
+      </c>
+      <c r="H46" s="39">
+        <v>50</v>
+      </c>
+      <c r="I46" s="37" t="s">
+        <v>628</v>
+      </c>
+      <c r="J46" s="37" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A47" s="43" t="s">
+        <v>630</v>
+      </c>
+      <c r="B47" s="44" t="s">
+        <v>582</v>
+      </c>
+      <c r="C47" s="44" t="s">
+        <v>631</v>
+      </c>
+      <c r="D47" s="44" t="s">
+        <v>578</v>
+      </c>
+      <c r="E47" s="46">
+        <v>30</v>
+      </c>
+      <c r="F47" s="46">
+        <v>0</v>
+      </c>
+      <c r="G47" s="47">
+        <v>118.4</v>
+      </c>
+      <c r="H47" s="46">
+        <v>70</v>
+      </c>
+      <c r="I47" s="44" t="s">
+        <v>632</v>
+      </c>
+      <c r="J47" s="44" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A48" s="36" t="s">
+        <v>634</v>
+      </c>
+      <c r="B48" s="37" t="s">
+        <v>582</v>
+      </c>
+      <c r="C48" s="37" t="s">
+        <v>578</v>
+      </c>
+      <c r="D48" s="37" t="s">
+        <v>635</v>
+      </c>
+      <c r="E48" s="39">
+        <v>0</v>
+      </c>
+      <c r="F48" s="39">
+        <v>30</v>
+      </c>
+      <c r="G48" s="40">
+        <v>102.4</v>
+      </c>
+      <c r="H48" s="39">
+        <v>60</v>
+      </c>
+      <c r="I48" s="37" t="s">
+        <v>636</v>
+      </c>
+      <c r="J48" s="37" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A49" s="43" t="s">
+        <v>638</v>
+      </c>
+      <c r="B49" s="44" t="s">
+        <v>582</v>
+      </c>
+      <c r="C49" s="44" t="s">
+        <v>639</v>
+      </c>
+      <c r="D49" s="44" t="s">
+        <v>578</v>
+      </c>
+      <c r="E49" s="46">
+        <v>30</v>
+      </c>
+      <c r="F49" s="46">
+        <v>0</v>
+      </c>
+      <c r="G49" s="47">
+        <v>102.4</v>
+      </c>
+      <c r="H49" s="46">
+        <v>80</v>
+      </c>
+      <c r="I49" s="44" t="s">
+        <v>640</v>
+      </c>
+      <c r="J49" s="44" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A50" s="36" t="s">
+        <v>642</v>
+      </c>
+      <c r="B50" s="37" t="s">
+        <v>643</v>
+      </c>
+      <c r="C50" s="37" t="s">
+        <v>644</v>
+      </c>
+      <c r="D50" s="37" t="s">
+        <v>645</v>
+      </c>
+      <c r="E50" s="39">
+        <v>30</v>
+      </c>
+      <c r="F50" s="39">
+        <v>30</v>
+      </c>
+      <c r="G50" s="40">
+        <v>116.4</v>
+      </c>
+      <c r="H50" s="39">
+        <v>70</v>
+      </c>
+      <c r="I50" s="37" t="s">
+        <v>646</v>
+      </c>
+      <c r="J50" s="37" t="s">
+        <v>647</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J12"/>
@@ -2260,7 +4963,7 @@
         <v>80</v>
       </c>
       <c r="F3" s="18">
-        <v>3650</v>
+        <v>500</v>
       </c>
       <c r="G3" s="14" t="s">
         <v>65</v>
@@ -2292,7 +4995,7 @@
         <v>15</v>
       </c>
       <c r="F4" s="24">
-        <v>2750</v>
+        <v>275</v>
       </c>
       <c r="G4" s="20" t="s">
         <v>65</v>
@@ -2516,7 +5219,7 @@
         <v>0</v>
       </c>
       <c r="F11" s="18">
-        <v>234000</v>
+        <v>173880</v>
       </c>
       <c r="G11" s="14" t="s">
         <v>98</v>
@@ -4391,14 +7094,14 @@
         <v>139006</v>
       </c>
       <c r="L3" s="18">
-        <v>3582500</v>
+        <v>691250</v>
       </c>
       <c r="M3" s="18">
-        <v>4350000</v>
+        <v>1000000</v>
       </c>
       <c r="N3" s="18">
         <f>M3-L3-K3</f>
-        <v>628494</v>
+        <v>169744</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4436,14 +7139,14 @@
         <v>139006</v>
       </c>
       <c r="L4" s="18">
-        <v>3582500</v>
-      </c>
-      <c r="M4" s="24">
-        <v>4350000</v>
+        <v>691250</v>
+      </c>
+      <c r="M4" s="18">
+        <v>1000000</v>
       </c>
       <c r="N4" s="18">
         <f t="shared" ref="N4:N12" si="0">M4-L4-K4</f>
-        <v>628494</v>
+        <v>169744</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4481,14 +7184,14 @@
         <v>139006</v>
       </c>
       <c r="L5" s="18">
-        <v>3582500</v>
+        <v>691250</v>
       </c>
       <c r="M5" s="18">
-        <v>4350000</v>
+        <v>1000000</v>
       </c>
       <c r="N5" s="18">
         <f t="shared" si="0"/>
-        <v>628494</v>
+        <v>169744</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4526,14 +7229,14 @@
         <v>139006</v>
       </c>
       <c r="L6" s="18">
-        <v>3582500</v>
-      </c>
-      <c r="M6" s="24">
-        <v>4350000</v>
+        <v>691250</v>
+      </c>
+      <c r="M6" s="18">
+        <v>1000000</v>
       </c>
       <c r="N6" s="18">
         <f t="shared" si="0"/>
-        <v>628494</v>
+        <v>169744</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4571,14 +7274,14 @@
         <v>139006</v>
       </c>
       <c r="L7" s="18">
-        <v>3582500</v>
+        <v>691250</v>
       </c>
       <c r="M7" s="18">
-        <v>4350000</v>
+        <v>1000000</v>
       </c>
       <c r="N7" s="18">
         <f t="shared" si="0"/>
-        <v>628494</v>
+        <v>169744</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4616,14 +7319,14 @@
         <v>139006</v>
       </c>
       <c r="L8" s="18">
-        <v>3582500</v>
-      </c>
-      <c r="M8" s="24">
-        <v>4350000</v>
+        <v>691250</v>
+      </c>
+      <c r="M8" s="18">
+        <v>1000000</v>
       </c>
       <c r="N8" s="18">
         <f t="shared" si="0"/>
-        <v>628494</v>
+        <v>169744</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4661,14 +7364,14 @@
         <v>139006</v>
       </c>
       <c r="L9" s="18">
-        <v>3582500</v>
+        <v>691250</v>
       </c>
       <c r="M9" s="18">
-        <v>4350000</v>
+        <v>1000000</v>
       </c>
       <c r="N9" s="18">
         <f t="shared" si="0"/>
-        <v>628494</v>
+        <v>169744</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4706,14 +7409,14 @@
         <v>139006</v>
       </c>
       <c r="L10" s="18">
-        <v>3582500</v>
-      </c>
-      <c r="M10" s="24">
-        <v>4350000</v>
+        <v>691250</v>
+      </c>
+      <c r="M10" s="18">
+        <v>1000000</v>
       </c>
       <c r="N10" s="18">
         <f t="shared" si="0"/>
-        <v>628494</v>
+        <v>169744</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4751,14 +7454,14 @@
         <v>139006</v>
       </c>
       <c r="L11" s="18">
-        <v>3582500</v>
+        <v>691250</v>
       </c>
       <c r="M11" s="18">
-        <v>4350000</v>
+        <v>1000000</v>
       </c>
       <c r="N11" s="18">
         <f t="shared" si="0"/>
-        <v>628494</v>
+        <v>169744</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4796,14 +7499,14 @@
         <v>139006</v>
       </c>
       <c r="L12" s="18">
-        <v>3582500</v>
-      </c>
-      <c r="M12" s="24">
-        <v>4350000</v>
+        <v>691250</v>
+      </c>
+      <c r="M12" s="18">
+        <v>1000000</v>
       </c>
       <c r="N12" s="18">
-        <f t="shared" si="0"/>
-        <v>628494</v>
+        <f>M12-L12-K12</f>
+        <v>169744</v>
       </c>
     </row>
   </sheetData>
@@ -4899,15 +7602,15 @@
       </c>
       <c r="I3" s="18">
         <f>F3*telemetri_produksi_scada!H3*master_bahan_baku!F11</f>
-        <v>5513508</v>
+        <v>4096960.56</v>
       </c>
       <c r="J3" s="18">
         <f>G3*biaya_siklus_hpp!N3</f>
-        <v>43994580</v>
+        <v>11882080</v>
       </c>
       <c r="K3" s="18">
         <f>SUM(H3:J3)</f>
-        <v>50845588</v>
+        <v>17316540.560000002</v>
       </c>
       <c r="L3" s="15" t="s">
         <v>377</v>
@@ -4940,15 +7643,15 @@
       </c>
       <c r="I4" s="24">
         <f>F4*telemetri_produksi_scada!H4*master_bahan_baku!F11</f>
-        <v>3198312</v>
+        <v>2376591.84</v>
       </c>
       <c r="J4" s="18">
         <f>G4*biaya_siklus_hpp!N4</f>
-        <v>25139760</v>
+        <v>6789760</v>
       </c>
       <c r="K4" s="18">
         <f t="shared" ref="K4:K12" si="0">SUM(H4:J4)</f>
-        <v>29102358</v>
+        <v>9930637.8399999999</v>
       </c>
       <c r="L4" s="21" t="s">
         <v>383</v>
@@ -4981,15 +7684,15 @@
       </c>
       <c r="I5" s="18">
         <f>F5*telemetri_produksi_scada!H5*master_bahan_baku!F11</f>
-        <v>3987945</v>
+        <v>2963349.9</v>
       </c>
       <c r="J5" s="18">
         <f>G5*biaya_siklus_hpp!N5</f>
-        <v>31424700</v>
+        <v>8487200</v>
       </c>
       <c r="K5" s="18">
         <f t="shared" si="0"/>
-        <v>36368002</v>
+        <v>12405906.9</v>
       </c>
       <c r="L5" s="15" t="s">
         <v>389</v>
@@ -5026,11 +7729,11 @@
       </c>
       <c r="J6" s="18">
         <f>G6*biaya_siklus_hpp!N6</f>
-        <v>18854820</v>
+        <v>5092320</v>
       </c>
       <c r="K6" s="18">
         <f t="shared" si="0"/>
-        <v>22302292</v>
+        <v>8539792</v>
       </c>
       <c r="L6" s="21" t="s">
         <v>394</v>
@@ -5063,15 +7766,15 @@
       </c>
       <c r="I7" s="18">
         <f>F7*telemetri_produksi_scada!H7*master_bahan_baku!F11</f>
-        <v>2380833</v>
+        <v>1769142.06</v>
       </c>
       <c r="J7" s="18">
         <f>G7*biaya_siklus_hpp!N7</f>
-        <v>18854820</v>
+        <v>5092320</v>
       </c>
       <c r="K7" s="18">
         <f t="shared" si="0"/>
-        <v>21808867</v>
+        <v>7434676.0600000005</v>
       </c>
       <c r="L7" s="15" t="s">
         <v>399</v>
@@ -5104,15 +7807,15 @@
       </c>
       <c r="I8" s="24">
         <f>F8*telemetri_produksi_scada!H8*master_bahan_baku!F11</f>
-        <v>1175499</v>
+        <v>873486.18</v>
       </c>
       <c r="J8" s="18">
         <f>G8*biaya_siklus_hpp!N8</f>
-        <v>9427410</v>
+        <v>2546160</v>
       </c>
       <c r="K8" s="18">
         <f t="shared" si="0"/>
-        <v>10889516</v>
+        <v>3706253.18</v>
       </c>
       <c r="L8" s="21" t="s">
         <v>404</v>
@@ -5145,15 +7848,15 @@
       </c>
       <c r="I9" s="18">
         <f>F9*telemetri_produksi_scada!H9*master_bahan_baku!F11</f>
-        <v>1607112</v>
+        <v>1194207.8400000001</v>
       </c>
       <c r="J9" s="18">
         <f>G9*biaya_siklus_hpp!N9</f>
-        <v>12569880</v>
+        <v>3394880</v>
       </c>
       <c r="K9" s="18">
         <f t="shared" si="0"/>
-        <v>14559135</v>
+        <v>4971230.84</v>
       </c>
       <c r="L9" s="15" t="s">
         <v>409</v>
@@ -5186,15 +7889,15 @@
       </c>
       <c r="I10" s="24">
         <f>F10*telemetri_produksi_scada!H10*master_bahan_baku!F11</f>
-        <v>3158532</v>
+        <v>2347032.2399999998</v>
       </c>
       <c r="J10" s="18">
         <f>G10*biaya_siklus_hpp!N10</f>
-        <v>25139760</v>
+        <v>6789760</v>
       </c>
       <c r="K10" s="18">
         <f t="shared" si="0"/>
-        <v>29062578</v>
+        <v>9901078.2400000002</v>
       </c>
       <c r="L10" s="21" t="s">
         <v>414</v>
@@ -5227,15 +7930,15 @@
       </c>
       <c r="I11" s="18">
         <f>F11*telemetri_produksi_scada!H11*master_bahan_baku!F11</f>
-        <v>1603134</v>
+        <v>1191251.8799999999</v>
       </c>
       <c r="J11" s="18">
         <f>G11*biaya_siklus_hpp!N11</f>
-        <v>12569880</v>
+        <v>3394880</v>
       </c>
       <c r="K11" s="18">
         <f t="shared" si="0"/>
-        <v>14555157</v>
+        <v>4968274.88</v>
       </c>
       <c r="L11" s="15" t="s">
         <v>419</v>
@@ -5268,15 +7971,15 @@
       </c>
       <c r="I12" s="24">
         <f>F12*telemetri_produksi_scada!H12*master_bahan_baku!F11</f>
-        <v>2486250</v>
+        <v>1847475</v>
       </c>
       <c r="J12" s="18">
         <f>G12*biaya_siklus_hpp!N12</f>
-        <v>31424700</v>
+        <v>8487200</v>
       </c>
       <c r="K12" s="18">
         <f t="shared" si="0"/>
-        <v>34866307</v>
+        <v>11290032</v>
       </c>
       <c r="L12" s="21" t="s">
         <v>424</v>

</xml_diff>